<commit_message>
Fix param doc --check line-ending mismatch between Windows and Cygwin Python
</commit_message>
<xml_diff>
--- a/doc/params/xplorer-params.xlsx
+++ b/doc/params/xplorer-params.xlsx
@@ -69814,7 +69814,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-13 20:23 UTC</t>
+          <t>2026-08-13 20:27 UTC</t>
         </is>
       </c>
     </row>
@@ -69826,7 +69826,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>d5934508a3</t>
+          <t>690fa484c6</t>
         </is>
       </c>
     </row>
@@ -69850,7 +69850,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Copter-4.6.1-150-gd5934508a3-dirty</t>
+          <t>xplorer-fw-v1.0.1-dirty</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Exclude git provenance from param doc --check comparison
</commit_message>
<xml_diff>
--- a/doc/params/xplorer-params.xlsx
+++ b/doc/params/xplorer-params.xlsx
@@ -69814,7 +69814,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-13 20:27 UTC</t>
+          <t>2026-08-13 20:34 UTC</t>
         </is>
       </c>
     </row>
@@ -69826,7 +69826,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>690fa484c6</t>
+          <t>2298c89a98</t>
         </is>
       </c>
     </row>

</xml_diff>